<commit_message>
updated readme with new todo
</commit_message>
<xml_diff>
--- a/config/sample_survey_responses1.xlsx
+++ b/config/sample_survey_responses1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cheun1/Projects/3strands-data-analysis/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76755900-769F-1A4E-8517-C2CDE6C5FBB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7397F8A0-09F7-F54C-8CB9-B7D3A087D05B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1900" yWindow="1900" windowWidth="27240" windowHeight="16180" xr2:uid="{C11B6343-5418-DF47-B0A8-461487D43C75}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="79">
   <si>
     <t>family_q1</t>
   </si>
@@ -270,13 +270,19 @@
   </si>
   <si>
     <t>Grace Lee</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>blah@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -295,6 +301,14 @@
       <sz val="10"/>
       <color rgb="FF434343"/>
       <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -335,18 +349,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="22" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -679,14 +696,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5067655C-5AA9-724C-A59B-AC7ECDDBA112}">
-  <dimension ref="A1:BI17"/>
+  <dimension ref="A1:BJ17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>58</v>
       </c>
@@ -696,182 +715,185 @@
       <c r="C1" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>46038.693692129629</v>
       </c>
@@ -881,26 +903,26 @@
       <c r="C2">
         <v>25</v>
       </c>
-      <c r="D2">
-        <v>4</v>
+      <c r="D2" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H2">
         <v>5</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>3</v>
@@ -909,127 +931,127 @@
         <v>3</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Z2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AA2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AB2">
         <v>1</v>
       </c>
       <c r="AC2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD2">
         <v>3</v>
       </c>
       <c r="AE2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG2">
         <v>4</v>
       </c>
       <c r="AH2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AI2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AJ2">
         <v>4</v>
       </c>
       <c r="AK2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AM2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AN2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AO2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AP2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AQ2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AS2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AT2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AV2">
         <v>2</v>
       </c>
       <c r="AW2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AZ2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BA2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BB2">
         <v>4</v>
@@ -1041,22 +1063,25 @@
         <v>4</v>
       </c>
       <c r="BE2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BF2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BG2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BH2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BI2">
+        <v>4</v>
+      </c>
+      <c r="BJ2">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>46038.705138888887</v>
       </c>
@@ -1066,65 +1091,65 @@
       <c r="C3">
         <v>28</v>
       </c>
-      <c r="D3">
-        <v>4</v>
+      <c r="D3" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3">
         <v>2</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J3">
         <v>2</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M3">
         <v>2</v>
       </c>
       <c r="N3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O3">
         <v>4</v>
       </c>
       <c r="P3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R3">
         <v>5</v>
       </c>
       <c r="S3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X3">
         <v>4</v>
@@ -1133,19 +1158,19 @@
         <v>4</v>
       </c>
       <c r="Z3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AB3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC3">
         <v>5</v>
       </c>
       <c r="AD3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE3">
         <v>1</v>
@@ -1157,91 +1182,94 @@
         <v>1</v>
       </c>
       <c r="AH3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AI3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AJ3">
         <v>3</v>
       </c>
       <c r="AK3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AL3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AM3">
         <v>3</v>
       </c>
       <c r="AN3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AO3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AP3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AQ3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AR3">
         <v>2</v>
       </c>
       <c r="AS3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AV3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AW3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AX3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AZ3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BA3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BB3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC3">
         <v>3</v>
       </c>
       <c r="BD3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BE3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BF3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BG3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BH3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BI3">
+        <v>1</v>
+      </c>
+      <c r="BJ3">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>46038.717627314814</v>
       </c>
@@ -1251,86 +1279,86 @@
       <c r="C4">
         <v>30</v>
       </c>
-      <c r="D4">
-        <v>2</v>
+      <c r="D4" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>2</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q4">
         <v>5</v>
       </c>
       <c r="R4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W4">
         <v>3</v>
       </c>
       <c r="X4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Z4">
         <v>2</v>
       </c>
       <c r="AA4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AB4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AD4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AE4">
         <v>4</v>
@@ -1345,16 +1373,16 @@
         <v>4</v>
       </c>
       <c r="AI4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AJ4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AK4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AL4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AM4">
         <v>1</v>
@@ -1366,67 +1394,70 @@
         <v>1</v>
       </c>
       <c r="AP4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AQ4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AS4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AT4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AU4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AV4">
         <v>3</v>
       </c>
       <c r="AW4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AX4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AY4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AZ4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BA4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BB4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BC4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BD4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BE4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BF4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BG4">
         <v>1</v>
       </c>
       <c r="BH4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BI4">
+        <v>2</v>
+      </c>
+      <c r="BJ4">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>46038.720995370371</v>
       </c>
@@ -1436,182 +1467,185 @@
       <c r="C5">
         <v>32</v>
       </c>
-      <c r="D5">
-        <v>4</v>
+      <c r="D5" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J5">
         <v>1</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N5">
         <v>2</v>
       </c>
       <c r="O5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R5">
         <v>1</v>
       </c>
       <c r="S5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Z5">
         <v>3</v>
       </c>
       <c r="AA5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AB5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AD5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG5">
         <v>1</v>
       </c>
       <c r="AH5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AI5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AJ5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AK5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AM5">
         <v>4</v>
       </c>
       <c r="AN5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AO5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AP5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AQ5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS5">
         <v>3</v>
       </c>
       <c r="AT5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AU5">
         <v>4</v>
       </c>
       <c r="AV5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AW5">
         <v>1</v>
       </c>
       <c r="AX5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AZ5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BA5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BB5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BC5">
         <v>1</v>
       </c>
       <c r="BD5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BE5">
         <v>2</v>
       </c>
       <c r="BF5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BG5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BH5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BI5">
+        <v>2</v>
+      </c>
+      <c r="BJ5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>46038.72446759259</v>
       </c>
@@ -1621,41 +1655,41 @@
       <c r="C6">
         <v>23</v>
       </c>
-      <c r="D6">
-        <v>4</v>
+      <c r="D6" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E6">
         <v>4</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N6">
         <v>1</v>
       </c>
       <c r="O6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P6">
         <v>3</v>
@@ -1664,43 +1698,43 @@
         <v>3</v>
       </c>
       <c r="R6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X6">
         <v>4</v>
       </c>
       <c r="Y6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Z6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AA6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AD6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AE6">
         <v>2</v>
@@ -1709,55 +1743,55 @@
         <v>2</v>
       </c>
       <c r="AG6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AI6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AJ6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AK6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AM6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AN6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AO6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AP6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AQ6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR6">
         <v>1</v>
       </c>
       <c r="AS6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AT6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU6">
         <v>3</v>
       </c>
       <c r="AV6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AW6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AX6">
         <v>3</v>
@@ -1766,37 +1800,40 @@
         <v>3</v>
       </c>
       <c r="AZ6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BA6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BB6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BC6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BD6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BE6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BF6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BG6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BH6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BI6">
+        <v>3</v>
+      </c>
+      <c r="BJ6">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>46038.725185185183</v>
       </c>
@@ -1806,98 +1843,98 @@
       <c r="C7">
         <v>25</v>
       </c>
-      <c r="D7">
-        <v>3</v>
+      <c r="D7" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H7">
         <v>4</v>
       </c>
       <c r="I7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7">
         <v>5</v>
       </c>
       <c r="K7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O7">
         <v>5</v>
       </c>
       <c r="P7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W7">
         <v>5</v>
       </c>
       <c r="X7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC7">
         <v>2</v>
       </c>
       <c r="AD7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF7">
         <v>2</v>
       </c>
       <c r="AG7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI7">
         <v>2</v>
@@ -1906,7 +1943,7 @@
         <v>2</v>
       </c>
       <c r="AK7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL7">
         <v>1</v>
@@ -1915,73 +1952,76 @@
         <v>1</v>
       </c>
       <c r="AN7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AP7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AQ7">
         <v>2</v>
       </c>
       <c r="AR7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AV7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AW7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AX7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AZ7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BA7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BB7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BC7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BD7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BE7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BF7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BG7">
         <v>2</v>
       </c>
       <c r="BH7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BI7">
+        <v>3</v>
+      </c>
+      <c r="BJ7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>46038.778634259259</v>
       </c>
@@ -1991,44 +2031,44 @@
       <c r="C8">
         <v>26</v>
       </c>
-      <c r="D8">
-        <v>2</v>
+      <c r="D8" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G8">
         <v>2</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q8">
         <v>4</v>
@@ -2037,100 +2077,100 @@
         <v>4</v>
       </c>
       <c r="S8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AA8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AB8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AF8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AG8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AH8">
         <v>2</v>
       </c>
       <c r="AI8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AJ8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AK8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AL8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AM8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AN8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AO8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AP8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AQ8">
         <v>2</v>
       </c>
       <c r="AR8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AT8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AV8">
         <v>5</v>
       </c>
       <c r="AW8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AX8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AY8">
         <v>5</v>
@@ -2139,34 +2179,37 @@
         <v>5</v>
       </c>
       <c r="BA8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BB8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BC8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BD8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BE8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BF8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BG8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BH8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BI8">
+        <v>4</v>
+      </c>
+      <c r="BJ8">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>46038.816759259258</v>
       </c>
@@ -2176,182 +2219,185 @@
       <c r="C9">
         <v>27</v>
       </c>
-      <c r="D9">
-        <v>1</v>
+      <c r="D9" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I9">
         <v>2</v>
       </c>
       <c r="J9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O9">
         <v>2</v>
       </c>
       <c r="P9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U9">
         <v>2</v>
       </c>
       <c r="V9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Z9">
         <v>5</v>
       </c>
       <c r="AA9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AB9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AF9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AG9">
         <v>4</v>
       </c>
       <c r="AH9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AI9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AK9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AL9">
         <v>1</v>
       </c>
       <c r="AM9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AN9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AO9">
         <v>3</v>
       </c>
       <c r="AP9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AQ9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AS9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT9">
         <v>1</v>
       </c>
       <c r="AU9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AV9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AX9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY9">
         <v>5</v>
       </c>
       <c r="AZ9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BA9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BB9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BC9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BD9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BE9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BF9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BH9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BI9">
+        <v>5</v>
+      </c>
+      <c r="BJ9">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>46038.907476851855</v>
       </c>
@@ -2361,8 +2407,8 @@
       <c r="C10">
         <v>28</v>
       </c>
-      <c r="D10">
-        <v>2</v>
+      <c r="D10" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E10">
         <v>2</v>
@@ -2371,97 +2417,97 @@
         <v>2</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S10">
         <v>5</v>
       </c>
       <c r="T10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="X10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AA10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AF10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AH10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AI10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AJ10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AK10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AL10">
         <v>1</v>
@@ -2470,73 +2516,76 @@
         <v>1</v>
       </c>
       <c r="AN10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AO10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AP10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AQ10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AR10">
         <v>3</v>
       </c>
       <c r="AS10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU10">
         <v>4</v>
       </c>
       <c r="AV10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AX10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AY10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AZ10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BA10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BB10">
         <v>4</v>
       </c>
       <c r="BC10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BD10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BE10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BF10">
         <v>5</v>
       </c>
       <c r="BG10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BH10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BI10">
+        <v>4</v>
+      </c>
+      <c r="BJ10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>46038.970868055556</v>
       </c>
@@ -2546,32 +2595,32 @@
       <c r="C11">
         <v>32</v>
       </c>
-      <c r="D11">
-        <v>4</v>
+      <c r="D11" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K11">
         <v>5</v>
       </c>
       <c r="L11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M11">
         <v>2</v>
@@ -2580,67 +2629,67 @@
         <v>2</v>
       </c>
       <c r="O11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S11">
         <v>3</v>
       </c>
       <c r="T11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X11">
         <v>2</v>
       </c>
       <c r="Y11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AA11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AB11">
         <v>5</v>
       </c>
       <c r="AC11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AD11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AH11">
         <v>2</v>
       </c>
       <c r="AI11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AJ11">
         <v>5</v>
@@ -2649,28 +2698,28 @@
         <v>5</v>
       </c>
       <c r="AL11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AM11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AN11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AO11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AP11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AQ11">
         <v>1</v>
       </c>
       <c r="AR11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AS11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AT11">
         <v>4</v>
@@ -2679,49 +2728,52 @@
         <v>4</v>
       </c>
       <c r="AV11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AW11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AX11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AY11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AZ11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BA11">
         <v>2</v>
       </c>
       <c r="BB11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BC11">
         <v>3</v>
       </c>
       <c r="BD11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BE11">
         <v>5</v>
       </c>
       <c r="BF11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BG11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BH11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BI11">
+        <v>2</v>
+      </c>
+      <c r="BJ11">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>46039.021736111114</v>
       </c>
@@ -2731,35 +2783,35 @@
       <c r="C12">
         <v>33</v>
       </c>
-      <c r="D12">
-        <v>4</v>
+      <c r="D12" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
       <c r="H12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I12">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N12">
         <v>1</v>
@@ -2768,16 +2820,16 @@
         <v>1</v>
       </c>
       <c r="P12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T12">
         <v>5</v>
@@ -2792,34 +2844,34 @@
         <v>5</v>
       </c>
       <c r="X12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Z12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AB12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AC12">
         <v>3</v>
       </c>
       <c r="AD12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AF12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH12">
         <v>1</v>
@@ -2828,73 +2880,73 @@
         <v>1</v>
       </c>
       <c r="AJ12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AK12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AO12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AP12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AQ12">
         <v>4</v>
       </c>
       <c r="AR12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AS12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AT12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AU12">
         <v>4</v>
       </c>
       <c r="AV12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AW12">
         <v>2</v>
       </c>
       <c r="AX12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AY12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AZ12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BA12">
         <v>4</v>
       </c>
       <c r="BB12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BC12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BD12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BE12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BF12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG12">
         <v>1</v>
@@ -2903,10 +2955,13 @@
         <v>1</v>
       </c>
       <c r="BI12">
+        <v>1</v>
+      </c>
+      <c r="BJ12">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>46039.247662037036</v>
       </c>
@@ -2916,41 +2971,41 @@
       <c r="C13">
         <v>30</v>
       </c>
-      <c r="D13">
-        <v>4</v>
+      <c r="D13" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H13">
         <v>5</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P13">
         <v>2</v>
@@ -2959,85 +3014,85 @@
         <v>2</v>
       </c>
       <c r="R13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T13">
         <v>5</v>
       </c>
       <c r="U13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V13">
         <v>1</v>
       </c>
       <c r="W13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AA13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AB13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD13">
         <v>3</v>
       </c>
       <c r="AE13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AF13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AG13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AH13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AK13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AL13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AM13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AO13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AP13">
         <v>5</v>
       </c>
       <c r="AQ13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AR13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AS13">
         <v>5</v>
@@ -3049,49 +3104,52 @@
         <v>5</v>
       </c>
       <c r="AV13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AW13">
         <v>2</v>
       </c>
       <c r="AX13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AZ13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BA13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BB13">
         <v>1</v>
       </c>
       <c r="BC13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BD13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BE13">
         <v>5</v>
       </c>
       <c r="BF13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BG13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BH13">
         <v>1</v>
       </c>
       <c r="BI13">
+        <v>1</v>
+      </c>
+      <c r="BJ13">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>46039.348680555559</v>
       </c>
@@ -3101,11 +3159,11 @@
       <c r="C14">
         <v>31</v>
       </c>
-      <c r="D14">
-        <v>4</v>
+      <c r="D14" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14">
         <v>2</v>
@@ -3114,55 +3172,55 @@
         <v>2</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I14">
         <v>3</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q14">
         <v>1</v>
       </c>
       <c r="R14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S14">
         <v>5</v>
       </c>
       <c r="T14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14">
         <v>3</v>
       </c>
       <c r="W14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="X14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y14">
         <v>2</v>
@@ -3174,79 +3232,79 @@
         <v>2</v>
       </c>
       <c r="AB14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC14">
         <v>3</v>
       </c>
       <c r="AD14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AF14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AG14">
         <v>1</v>
       </c>
       <c r="AH14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AI14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AJ14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AK14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AL14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AM14">
         <v>5</v>
       </c>
       <c r="AN14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AO14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AP14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AT14">
         <v>4</v>
       </c>
       <c r="AU14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AV14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AW14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AX14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AY14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AZ14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BA14">
         <v>3</v>
@@ -3258,25 +3316,28 @@
         <v>3</v>
       </c>
       <c r="BD14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BE14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BF14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BG14">
         <v>4</v>
       </c>
       <c r="BH14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BI14">
+        <v>1</v>
+      </c>
+      <c r="BJ14">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>46039.44090277778</v>
       </c>
@@ -3286,140 +3347,140 @@
       <c r="C15">
         <v>34</v>
       </c>
-      <c r="D15">
-        <v>3</v>
+      <c r="D15" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E15">
         <v>3</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15">
         <v>3</v>
       </c>
       <c r="L15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M15">
         <v>5</v>
       </c>
       <c r="N15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R15">
         <v>5</v>
       </c>
       <c r="S15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="T15">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X15">
         <v>2</v>
       </c>
       <c r="Y15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AB15">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AC15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF15">
         <v>1</v>
       </c>
       <c r="AG15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AI15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AJ15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AK15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AL15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AM15">
         <v>1</v>
       </c>
       <c r="AN15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AP15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AR15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AS15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AT15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AU15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AV15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW15">
         <v>3</v>
@@ -3431,37 +3492,40 @@
         <v>3</v>
       </c>
       <c r="AZ15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BA15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BB15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BC15">
         <v>2</v>
       </c>
       <c r="BD15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BE15">
         <v>3</v>
       </c>
       <c r="BF15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG15">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BH15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BI15">
+        <v>4</v>
+      </c>
+      <c r="BJ15">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>46039.44740740741</v>
       </c>
@@ -3471,182 +3535,185 @@
       <c r="C16">
         <v>26</v>
       </c>
-      <c r="D16">
-        <v>1</v>
+      <c r="D16" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I16">
         <v>1</v>
       </c>
       <c r="J16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AA16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AB16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC16">
         <v>2</v>
       </c>
       <c r="AD16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE16">
         <v>3</v>
       </c>
       <c r="AF16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AG16">
         <v>5</v>
       </c>
       <c r="AH16">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AI16">
         <v>1</v>
       </c>
       <c r="AJ16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AK16">
         <v>5</v>
       </c>
       <c r="AL16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AM16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AN16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AO16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AP16">
         <v>3</v>
       </c>
       <c r="AQ16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AR16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AT16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AU16">
         <v>4</v>
       </c>
       <c r="AV16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AW16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AX16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AY16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AZ16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BA16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BB16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BC16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BD16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BE16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BF16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BG16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BH16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BI16">
+        <v>2</v>
+      </c>
+      <c r="BJ16">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>46039.492442129631</v>
       </c>
@@ -3656,86 +3723,86 @@
       <c r="C17">
         <v>30</v>
       </c>
-      <c r="D17">
-        <v>3</v>
+      <c r="D17" s="4" t="s">
+        <v>78</v>
       </c>
       <c r="E17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q17">
         <v>3</v>
       </c>
       <c r="R17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T17">
         <v>2</v>
       </c>
       <c r="U17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V17">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="X17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Z17">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AA17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AB17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AC17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AD17">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE17">
         <v>1</v>
@@ -3744,73 +3811,73 @@
         <v>1</v>
       </c>
       <c r="AG17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH17">
         <v>3</v>
       </c>
       <c r="AI17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AJ17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AK17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AL17">
         <v>4</v>
       </c>
       <c r="AM17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AN17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AO17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AP17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AQ17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AS17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AT17">
         <v>3</v>
       </c>
       <c r="AU17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AV17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AW17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AX17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AY17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AZ17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BA17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BB17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BC17">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BD17">
         <v>5</v>
@@ -3819,19 +3886,26 @@
         <v>5</v>
       </c>
       <c r="BF17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BG17">
         <v>3</v>
       </c>
       <c r="BH17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BI17">
+        <v>2</v>
+      </c>
+      <c r="BJ17">
         <v>4</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{0C7146F2-09C7-3E4D-984A-9339CEFC558B}"/>
+    <hyperlink ref="D3:D17" r:id="rId2" display="blah@gmail.com" xr:uid="{18D22626-4309-B247-8481-D6666B4E5E3D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
implemented having four rounds and matching between people of diff gender only
</commit_message>
<xml_diff>
--- a/config/sample_survey_responses1.xlsx
+++ b/config/sample_survey_responses1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cheun1/Projects/3strands-data-analysis/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7397F8A0-09F7-F54C-8CB9-B7D3A087D05B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6556425E-97B8-484A-8884-5BA876292AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1900" yWindow="1900" windowWidth="27240" windowHeight="16180" xr2:uid="{C11B6343-5418-DF47-B0A8-461487D43C75}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="82">
   <si>
     <t>family_q1</t>
   </si>
@@ -276,6 +276,15 @@
   </si>
   <si>
     <t>blah@gmail.com</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>F</t>
   </si>
 </sst>
 </file>
@@ -696,16 +705,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5067655C-5AA9-724C-A59B-AC7ECDDBA112}">
-  <dimension ref="A1:BJ17"/>
+  <dimension ref="A1:BK17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>58</v>
       </c>
@@ -718,182 +727,185 @@
       <c r="D1" t="s">
         <v>77</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>46038.693692129629</v>
       </c>
@@ -906,26 +918,26 @@
       <c r="D2" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E2">
-        <v>4</v>
+      <c r="E2" t="s">
+        <v>80</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I2">
         <v>5</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L2">
         <v>3</v>
@@ -934,127 +946,127 @@
         <v>3</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="X2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Z2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AB2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AC2">
         <v>1</v>
       </c>
       <c r="AD2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE2">
         <v>3</v>
       </c>
       <c r="AF2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AH2">
         <v>4</v>
       </c>
       <c r="AI2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AJ2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AK2">
         <v>4</v>
       </c>
       <c r="AL2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AM2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AO2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AP2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AQ2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AR2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AT2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AU2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AV2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AW2">
         <v>2</v>
       </c>
       <c r="AX2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AZ2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BA2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BB2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BC2">
         <v>4</v>
@@ -1066,22 +1078,25 @@
         <v>4</v>
       </c>
       <c r="BF2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BG2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BH2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BI2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BJ2">
+        <v>4</v>
+      </c>
+      <c r="BK2">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>46038.705138888887</v>
       </c>
@@ -1094,65 +1109,65 @@
       <c r="D3" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E3">
-        <v>4</v>
+      <c r="E3" t="s">
+        <v>81</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G3">
         <v>2</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K3">
         <v>2</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N3">
         <v>2</v>
       </c>
       <c r="O3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P3">
         <v>4</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S3">
         <v>5</v>
       </c>
       <c r="T3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y3">
         <v>4</v>
@@ -1161,19 +1176,19 @@
         <v>4</v>
       </c>
       <c r="AA3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AD3">
         <v>5</v>
       </c>
       <c r="AE3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF3">
         <v>1</v>
@@ -1185,91 +1200,94 @@
         <v>1</v>
       </c>
       <c r="AI3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AJ3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AK3">
         <v>3</v>
       </c>
       <c r="AL3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AN3">
         <v>3</v>
       </c>
       <c r="AO3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AP3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AQ3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AR3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AS3">
         <v>2</v>
       </c>
       <c r="AT3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AV3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AW3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AX3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AY3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AZ3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BA3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BB3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BC3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BD3">
         <v>3</v>
       </c>
       <c r="BE3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BG3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BH3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BI3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BJ3">
+        <v>1</v>
+      </c>
+      <c r="BK3">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>46038.717627314814</v>
       </c>
@@ -1282,86 +1300,86 @@
       <c r="D4" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E4">
-        <v>2</v>
+      <c r="E4" t="s">
+        <v>81</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4">
         <v>2</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R4">
         <v>5</v>
       </c>
       <c r="S4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X4">
         <v>3</v>
       </c>
       <c r="Y4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Z4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AA4">
         <v>2</v>
       </c>
       <c r="AB4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AC4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AD4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AF4">
         <v>4</v>
@@ -1376,16 +1394,16 @@
         <v>4</v>
       </c>
       <c r="AJ4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AK4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AL4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AM4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AN4">
         <v>1</v>
@@ -1397,67 +1415,70 @@
         <v>1</v>
       </c>
       <c r="AQ4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AR4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AT4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AU4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AV4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AW4">
         <v>3</v>
       </c>
       <c r="AX4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AY4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AZ4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BA4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BB4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BC4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BD4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BE4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BG4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BH4">
         <v>1</v>
       </c>
       <c r="BI4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BJ4">
+        <v>2</v>
+      </c>
+      <c r="BK4">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>46038.720995370371</v>
       </c>
@@ -1470,182 +1491,185 @@
       <c r="D5" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E5">
-        <v>4</v>
+      <c r="E5" t="s">
+        <v>80</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O5">
         <v>2</v>
       </c>
       <c r="P5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="S5">
         <v>1</v>
       </c>
       <c r="T5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AA5">
         <v>3</v>
       </c>
       <c r="AB5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AD5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AE5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AF5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH5">
         <v>1</v>
       </c>
       <c r="AI5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AJ5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AK5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AL5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AM5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AN5">
         <v>4</v>
       </c>
       <c r="AO5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AP5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AQ5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT5">
         <v>3</v>
       </c>
       <c r="AU5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AV5">
         <v>4</v>
       </c>
       <c r="AW5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AX5">
         <v>1</v>
       </c>
       <c r="AY5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AZ5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BB5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BC5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BD5">
         <v>1</v>
       </c>
       <c r="BE5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BF5">
         <v>2</v>
       </c>
       <c r="BG5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BH5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BI5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BJ5">
+        <v>2</v>
+      </c>
+      <c r="BK5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>46038.72446759259</v>
       </c>
@@ -1658,41 +1682,41 @@
       <c r="D6" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E6">
-        <v>4</v>
+      <c r="E6" t="s">
+        <v>81</v>
       </c>
       <c r="F6">
         <v>4</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6">
         <v>5</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O6">
         <v>1</v>
       </c>
       <c r="P6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q6">
         <v>3</v>
@@ -1701,43 +1725,43 @@
         <v>3</v>
       </c>
       <c r="S6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y6">
         <v>4</v>
       </c>
       <c r="Z6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AA6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AB6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AF6">
         <v>2</v>
@@ -1746,55 +1770,55 @@
         <v>2</v>
       </c>
       <c r="AH6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AJ6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AK6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AL6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AM6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AN6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AO6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AP6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AQ6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS6">
         <v>1</v>
       </c>
       <c r="AT6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AV6">
         <v>3</v>
       </c>
       <c r="AW6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AX6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AY6">
         <v>3</v>
@@ -1803,37 +1827,40 @@
         <v>3</v>
       </c>
       <c r="BA6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BB6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BC6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BD6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BE6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BF6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BG6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BH6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BI6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BJ6">
+        <v>3</v>
+      </c>
+      <c r="BK6">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>46038.725185185183</v>
       </c>
@@ -1846,98 +1873,98 @@
       <c r="D7" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E7">
-        <v>3</v>
+      <c r="E7" t="s">
+        <v>80</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <v>4</v>
       </c>
       <c r="J7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K7">
         <v>5</v>
       </c>
       <c r="L7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P7">
         <v>5</v>
       </c>
       <c r="Q7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="X7">
         <v>5</v>
       </c>
       <c r="Y7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Z7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AA7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD7">
         <v>2</v>
       </c>
       <c r="AE7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG7">
         <v>2</v>
       </c>
       <c r="AH7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AJ7">
         <v>2</v>
@@ -1946,7 +1973,7 @@
         <v>2</v>
       </c>
       <c r="AL7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM7">
         <v>1</v>
@@ -1955,73 +1982,76 @@
         <v>1</v>
       </c>
       <c r="AO7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AP7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AQ7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AR7">
         <v>2</v>
       </c>
       <c r="AS7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AU7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AW7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AX7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AY7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AZ7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BA7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BB7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BC7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BD7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BE7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BF7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BG7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BH7">
         <v>2</v>
       </c>
       <c r="BI7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BJ7">
+        <v>3</v>
+      </c>
+      <c r="BK7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>46038.778634259259</v>
       </c>
@@ -2034,44 +2064,44 @@
       <c r="D8" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E8">
-        <v>2</v>
+      <c r="E8" t="s">
+        <v>80</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R8">
         <v>4</v>
@@ -2080,100 +2110,100 @@
         <v>4</v>
       </c>
       <c r="T8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Z8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AB8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AF8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AG8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AH8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AI8">
         <v>2</v>
       </c>
       <c r="AJ8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AK8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AL8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AM8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AN8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AO8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AP8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AQ8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR8">
         <v>2</v>
       </c>
       <c r="AS8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AU8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AW8">
         <v>5</v>
       </c>
       <c r="AX8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AY8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AZ8">
         <v>5</v>
@@ -2182,34 +2212,37 @@
         <v>5</v>
       </c>
       <c r="BB8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BC8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BD8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BE8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BF8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BG8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BH8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BI8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BJ8">
+        <v>4</v>
+      </c>
+      <c r="BK8">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>46038.816759259258</v>
       </c>
@@ -2222,182 +2255,185 @@
       <c r="D9" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E9">
-        <v>1</v>
+      <c r="E9" t="s">
+        <v>81</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J9">
         <v>2</v>
       </c>
       <c r="K9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P9">
         <v>2</v>
       </c>
       <c r="Q9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V9">
         <v>2</v>
       </c>
       <c r="W9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AA9">
         <v>5</v>
       </c>
       <c r="AB9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AF9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AH9">
         <v>4</v>
       </c>
       <c r="AI9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AJ9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AK9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AL9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AM9">
         <v>1</v>
       </c>
       <c r="AN9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AO9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AP9">
         <v>3</v>
       </c>
       <c r="AQ9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AR9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AT9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AU9">
         <v>1</v>
       </c>
       <c r="AV9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AW9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AX9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AZ9">
         <v>5</v>
       </c>
       <c r="BA9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BB9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BC9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BD9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BE9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BG9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BH9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BI9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BJ9">
+        <v>5</v>
+      </c>
+      <c r="BK9">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>46038.907476851855</v>
       </c>
@@ -2410,8 +2446,8 @@
       <c r="D10" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E10">
-        <v>2</v>
+      <c r="E10" t="s">
+        <v>81</v>
       </c>
       <c r="F10">
         <v>2</v>
@@ -2420,97 +2456,97 @@
         <v>2</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="T10">
         <v>5</v>
       </c>
       <c r="U10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Y10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Z10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AA10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AB10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AD10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AG10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AH10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AI10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AJ10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AK10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AL10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM10">
         <v>1</v>
@@ -2519,73 +2555,76 @@
         <v>1</v>
       </c>
       <c r="AO10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AP10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AQ10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AR10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AS10">
         <v>3</v>
       </c>
       <c r="AT10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AU10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AV10">
         <v>4</v>
       </c>
       <c r="AW10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AX10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AY10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AZ10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BA10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BB10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BC10">
         <v>4</v>
       </c>
       <c r="BD10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BE10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BF10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BG10">
         <v>5</v>
       </c>
       <c r="BH10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BI10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BJ10">
+        <v>4</v>
+      </c>
+      <c r="BK10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>46038.970868055556</v>
       </c>
@@ -2598,32 +2637,32 @@
       <c r="D11" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E11">
-        <v>4</v>
+      <c r="E11" t="s">
+        <v>80</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L11">
         <v>5</v>
       </c>
       <c r="M11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N11">
         <v>2</v>
@@ -2632,67 +2671,67 @@
         <v>2</v>
       </c>
       <c r="P11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T11">
         <v>3</v>
       </c>
       <c r="U11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="X11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y11">
         <v>2</v>
       </c>
       <c r="Z11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AA11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AB11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC11">
         <v>5</v>
       </c>
       <c r="AD11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AE11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AI11">
         <v>2</v>
       </c>
       <c r="AJ11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AK11">
         <v>5</v>
@@ -2701,28 +2740,28 @@
         <v>5</v>
       </c>
       <c r="AM11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AN11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AO11">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AP11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AQ11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AR11">
         <v>1</v>
       </c>
       <c r="AS11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AT11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AU11">
         <v>4</v>
@@ -2731,49 +2770,52 @@
         <v>4</v>
       </c>
       <c r="AW11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AX11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AZ11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BA11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BB11">
         <v>2</v>
       </c>
       <c r="BC11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BD11">
         <v>3</v>
       </c>
       <c r="BE11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BF11">
         <v>5</v>
       </c>
       <c r="BG11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BH11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BI11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BJ11">
+        <v>2</v>
+      </c>
+      <c r="BK11">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>46039.021736111114</v>
       </c>
@@ -2786,35 +2828,35 @@
       <c r="D12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E12">
-        <v>4</v>
+      <c r="E12" t="s">
+        <v>81</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J12">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O12">
         <v>1</v>
@@ -2823,16 +2865,16 @@
         <v>1</v>
       </c>
       <c r="Q12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U12">
         <v>5</v>
@@ -2847,34 +2889,34 @@
         <v>5</v>
       </c>
       <c r="Y12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Z12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AA12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AD12">
         <v>3</v>
       </c>
       <c r="AE12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AG12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AI12">
         <v>1</v>
@@ -2883,73 +2925,73 @@
         <v>1</v>
       </c>
       <c r="AK12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AL12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AM12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AN12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AO12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AP12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AQ12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AR12">
         <v>4</v>
       </c>
       <c r="AS12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AT12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AU12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AV12">
         <v>4</v>
       </c>
       <c r="AW12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AX12">
         <v>2</v>
       </c>
       <c r="AY12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AZ12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BA12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BB12">
         <v>4</v>
       </c>
       <c r="BC12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BD12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BE12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BF12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BG12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BH12">
         <v>1</v>
@@ -2958,10 +3000,13 @@
         <v>1</v>
       </c>
       <c r="BJ12">
+        <v>1</v>
+      </c>
+      <c r="BK12">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>46039.247662037036</v>
       </c>
@@ -2974,41 +3019,41 @@
       <c r="D13" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E13">
-        <v>4</v>
+      <c r="E13" t="s">
+        <v>80</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I13">
         <v>5</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q13">
         <v>2</v>
@@ -3017,85 +3062,85 @@
         <v>2</v>
       </c>
       <c r="S13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U13">
         <v>5</v>
       </c>
       <c r="V13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W13">
         <v>1</v>
       </c>
       <c r="X13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AA13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AB13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AC13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AD13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE13">
         <v>3</v>
       </c>
       <c r="AF13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AH13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AI13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AK13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AL13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AN13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AO13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AP13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AQ13">
         <v>5</v>
       </c>
       <c r="AR13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AS13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AT13">
         <v>5</v>
@@ -3107,49 +3152,52 @@
         <v>5</v>
       </c>
       <c r="AW13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AX13">
         <v>2</v>
       </c>
       <c r="AY13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AZ13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BA13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BB13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="BC13">
         <v>1</v>
       </c>
       <c r="BD13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BE13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BF13">
         <v>5</v>
       </c>
       <c r="BG13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BH13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BI13">
         <v>1</v>
       </c>
       <c r="BJ13">
+        <v>1</v>
+      </c>
+      <c r="BK13">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>46039.348680555559</v>
       </c>
@@ -3162,11 +3210,11 @@
       <c r="D14" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E14">
-        <v>4</v>
+      <c r="E14" t="s">
+        <v>80</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G14">
         <v>2</v>
@@ -3175,55 +3223,55 @@
         <v>2</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14">
         <v>3</v>
       </c>
       <c r="K14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R14">
         <v>1</v>
       </c>
       <c r="S14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="T14">
         <v>5</v>
       </c>
       <c r="U14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W14">
         <v>3</v>
       </c>
       <c r="X14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Z14">
         <v>2</v>
@@ -3235,79 +3283,79 @@
         <v>2</v>
       </c>
       <c r="AC14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD14">
         <v>3</v>
       </c>
       <c r="AE14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AF14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AH14">
         <v>1</v>
       </c>
       <c r="AI14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AJ14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AK14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AL14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AN14">
         <v>5</v>
       </c>
       <c r="AO14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AP14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AQ14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AU14">
         <v>4</v>
       </c>
       <c r="AV14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AW14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AX14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AY14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AZ14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="BA14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BB14">
         <v>3</v>
@@ -3319,25 +3367,28 @@
         <v>3</v>
       </c>
       <c r="BE14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BF14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BG14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BH14">
         <v>4</v>
       </c>
       <c r="BI14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BJ14">
+        <v>1</v>
+      </c>
+      <c r="BK14">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>46039.44090277778</v>
       </c>
@@ -3350,140 +3401,140 @@
       <c r="D15" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E15">
-        <v>3</v>
+      <c r="E15" t="s">
+        <v>81</v>
       </c>
       <c r="F15">
         <v>3</v>
       </c>
       <c r="G15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L15">
         <v>3</v>
       </c>
       <c r="M15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N15">
         <v>5</v>
       </c>
       <c r="O15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S15">
         <v>5</v>
       </c>
       <c r="T15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U15">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y15">
         <v>2</v>
       </c>
       <c r="Z15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AC15">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AD15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG15">
         <v>1</v>
       </c>
       <c r="AH15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AJ15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AK15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AL15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AM15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AN15">
         <v>1</v>
       </c>
       <c r="AO15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AP15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AQ15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AR15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AS15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AT15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AU15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AV15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AW15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AX15">
         <v>3</v>
@@ -3495,37 +3546,40 @@
         <v>3</v>
       </c>
       <c r="BA15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BB15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BC15">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BD15">
         <v>2</v>
       </c>
       <c r="BE15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BF15">
         <v>3</v>
       </c>
       <c r="BG15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BH15">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BI15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BJ15">
+        <v>4</v>
+      </c>
+      <c r="BK15">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>46039.44740740741</v>
       </c>
@@ -3538,182 +3592,185 @@
       <c r="D16" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E16">
-        <v>1</v>
+      <c r="E16" t="s">
+        <v>80</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J16">
         <v>1</v>
       </c>
       <c r="K16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AB16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD16">
         <v>2</v>
       </c>
       <c r="AE16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF16">
         <v>3</v>
       </c>
       <c r="AG16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AH16">
         <v>5</v>
       </c>
       <c r="AI16">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AJ16">
         <v>1</v>
       </c>
       <c r="AK16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AL16">
         <v>5</v>
       </c>
       <c r="AM16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AO16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AP16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AQ16">
         <v>3</v>
       </c>
       <c r="AR16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AS16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AT16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AU16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AV16">
         <v>4</v>
       </c>
       <c r="AW16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AX16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AZ16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BA16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BB16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BC16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BD16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BE16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BF16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BG16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BH16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="BI16">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="BJ16">
+        <v>2</v>
+      </c>
+      <c r="BK16">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:63" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>46039.492442129631</v>
       </c>
@@ -3726,86 +3783,86 @@
       <c r="D17" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E17">
-        <v>3</v>
+      <c r="E17" t="s">
+        <v>81</v>
       </c>
       <c r="F17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R17">
         <v>3</v>
       </c>
       <c r="S17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U17">
         <v>2</v>
       </c>
       <c r="V17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W17">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Z17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA17">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AB17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AD17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE17">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF17">
         <v>1</v>
@@ -3814,73 +3871,73 @@
         <v>1</v>
       </c>
       <c r="AH17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AI17">
         <v>3</v>
       </c>
       <c r="AJ17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AK17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AL17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AM17">
         <v>4</v>
       </c>
       <c r="AN17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AO17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AP17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AQ17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AT17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AU17">
         <v>3</v>
       </c>
       <c r="AV17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AW17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AX17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AY17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AZ17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BA17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BB17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BC17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BD17">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BE17">
         <v>5</v>
@@ -3889,15 +3946,18 @@
         <v>5</v>
       </c>
       <c r="BG17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BH17">
         <v>3</v>
       </c>
       <c r="BI17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BJ17">
+        <v>2</v>
+      </c>
+      <c r="BK17">
         <v>4</v>
       </c>
     </row>

</xml_diff>